<commit_message>
Initial commit - Cucumber framework with Extent & Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varun.bantia\eclipse-workspace\BBD-POM_FRAMEWORK\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2559C328-EC83-42F3-BC11-8D8C3593BE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8695FF7-2781-4BAE-A158-DAE65B0CD6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,10 +60,10 @@
     <t>wrongpass</t>
   </si>
   <si>
-    <t>Your ldkgmpr</t>
-  </si>
-  <si>
-    <t>d[pgk</t>
+    <t>Your username is invalid!</t>
+  </si>
+  <si>
+    <t>Your password is invalid!</t>
   </si>
 </sst>
 </file>
@@ -490,7 +490,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -504,7 +504,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>

</xml_diff>